<commit_message>
Integrated SMTP & IMAP With the Multi Juridictions and alway refactored the along with fixing some Bugs
</commit_message>
<xml_diff>
--- a/frontend/public/templates/employee-import-template.xlsx
+++ b/frontend/public/templates/employee-import-template.xlsx
@@ -426,30 +426,30 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD2"/>
+  <dimension ref="A1:AG2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="23" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="19" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
-    <col width="9" customWidth="1" min="11" max="11"/>
-    <col width="18" customWidth="1" min="12" max="12"/>
-    <col width="16" customWidth="1" min="13" max="13"/>
-    <col width="9" customWidth="1" min="14" max="14"/>
-    <col width="15" customWidth="1" min="15" max="15"/>
-    <col width="10" customWidth="1" min="16" max="16"/>
-    <col width="19" customWidth="1" min="17" max="17"/>
-    <col width="17" customWidth="1" min="18" max="18"/>
-    <col width="20" customWidth="1" min="19" max="19"/>
-    <col width="11" customWidth="1" min="20" max="20"/>
-    <col width="16" customWidth="1" min="21" max="21"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="19" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="9" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="9" customWidth="1" min="15" max="15"/>
+    <col width="15" customWidth="1" min="16" max="16"/>
+    <col width="9" customWidth="1" min="17" max="17"/>
+    <col width="10" customWidth="1" min="18" max="18"/>
+    <col width="19" customWidth="1" min="19" max="19"/>
+    <col width="17" customWidth="1" min="20" max="20"/>
+    <col width="11" customWidth="1" min="21" max="21"/>
     <col width="14" customWidth="1" min="22" max="22"/>
     <col width="11" customWidth="1" min="23" max="23"/>
     <col width="22" customWidth="1" min="24" max="24"/>
@@ -458,115 +458,118 @@
     <col width="14" customWidth="1" min="27" max="27"/>
     <col width="10" customWidth="1" min="28" max="28"/>
     <col width="10" customWidth="1" min="29" max="29"/>
-    <col width="10" customWidth="1" min="30" max="30"/>
+    <col width="13" customWidth="1" min="30" max="30"/>
+    <col width="15" customWidth="1" min="31" max="31"/>
+    <col width="22" customWidth="1" min="32" max="32"/>
+    <col width="14" customWidth="1" min="33" max="33"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>Employee ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>First Name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Last Name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Password</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Phone</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Job Title</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Department</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Designation</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Reporting Manager</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Employment Type</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Date of Joining</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Date of Birth</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Gender</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Basic Salary</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>HRA</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>CTC</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Work Email</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Personal Email</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>Confirmation Date</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
-          <t>Business Unit</t>
-        </is>
-      </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Division</t>
@@ -609,116 +612,131 @@
       </c>
       <c r="AD1" s="1" t="inlineStr">
         <is>
-          <t>Address</t>
+          <t>PAN Number</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>UAN</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>Bank Account Number</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>IFSC Code</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>ZO0001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>John</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Doe</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>john.doe@example.com</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>Pass@1234</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>+91-9876543210</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>Software Engineer</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>Engineering</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>Senior Developer</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>Jane Smith</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>Full Time</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>2024-01-15</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>1995-06-15</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>Male</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>75000</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>180000</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
         <is>
           <t>1200000</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="S2" t="inlineStr">
         <is>
           <t>john@company.com</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="T2" t="inlineStr">
         <is>
           <t>john@gmail.com</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>2024-07-15</t>
-        </is>
-      </c>
-      <c r="T2" t="inlineStr">
+      <c r="U2" t="inlineStr">
         <is>
           <t>ZoikoOne</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>Enterprise</t>
-        </is>
-      </c>
       <c r="V2" t="inlineStr">
         <is>
           <t>Engineering</t>
@@ -759,7 +777,26 @@
           <t>400001</t>
         </is>
       </c>
-      <c r="AD2" t="inlineStr"/>
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t>ABCDE1234F</t>
+        </is>
+      </c>
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>101234567890</t>
+        </is>
+      </c>
+      <c r="AF2" t="inlineStr">
+        <is>
+          <t>12345678901</t>
+        </is>
+      </c>
+      <c r="AG2" t="inlineStr">
+        <is>
+          <t>SBIN0001234</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>